<commit_message>
add unique variable length
</commit_message>
<xml_diff>
--- a/4_Documentation/codebook.xlsx
+++ b/4_Documentation/codebook.xlsx
@@ -425,13 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>variable_name</t>
+          <t>var_name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -441,10 +441,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>encoded_as</t>
+          <t>level</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>var_length</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
@@ -458,7 +463,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>761</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -472,7 +480,10 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>124</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -486,7 +497,10 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -500,7 +514,10 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -514,7 +531,10 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -528,7 +548,10 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -542,7 +565,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -556,7 +582,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -570,7 +599,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -584,7 +616,10 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -598,7 +633,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -612,7 +650,10 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -626,7 +667,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -640,7 +684,10 @@
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -654,7 +701,10 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -668,7 +718,10 @@
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="n">
+        <v>1331</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -682,7 +735,10 @@
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -696,7 +752,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
+      <c r="D19" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -710,7 +769,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -724,7 +786,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="n">
+        <v>1798</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -738,7 +803,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="n">
+        <v>1761</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -752,7 +820,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="n">
+        <v>12</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -766,7 +837,10 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
+      <c r="D24" t="n">
+        <v>47</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -780,7 +854,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="n">
+        <v>19</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -794,7 +871,10 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="n">
+        <v>292</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -808,7 +888,10 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -822,7 +905,10 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -836,7 +922,10 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -850,7 +939,10 @@
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -864,7 +956,10 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -878,7 +973,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
+      <c r="D32" t="n">
+        <v>7</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -892,7 +990,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
+      <c r="D33" t="n">
+        <v>327</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -906,7 +1007,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -920,7 +1024,10 @@
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -934,7 +1041,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
+      <c r="D36" t="n">
+        <v>11</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -948,7 +1058,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -962,7 +1075,10 @@
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -976,7 +1092,10 @@
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -990,7 +1109,10 @@
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1004,7 +1126,10 @@
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1018,7 +1143,10 @@
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1032,7 +1160,10 @@
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1046,7 +1177,10 @@
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1060,7 +1194,10 @@
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
+      <c r="D45" t="n">
+        <v>127</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1074,7 +1211,10 @@
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr">
+      <c r="D46" t="n">
+        <v>125</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1088,7 +1228,10 @@
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr">
+      <c r="D47" t="n">
+        <v>126</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1102,7 +1245,10 @@
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr">
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1116,7 +1262,10 @@
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr">
+      <c r="D49" t="n">
+        <v>304</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1130,7 +1279,10 @@
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr">
+      <c r="D50" t="n">
+        <v>15</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1144,7 +1296,10 @@
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr">
+      <c r="D51" t="n">
+        <v>761</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1158,7 +1313,10 @@
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr">
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1172,7 +1330,10 @@
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr">
+      <c r="D53" t="n">
+        <v>138</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1186,7 +1347,10 @@
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr">
+      <c r="D54" t="n">
+        <v>144</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1200,7 +1364,10 @@
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr">
+      <c r="D55" t="n">
+        <v>124</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1214,7 +1381,10 @@
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr">
+      <c r="D56" t="n">
+        <v>23</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>ACLED_all_ZCTA_nb.csv</t>
         </is>
@@ -1228,7 +1398,10 @@
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr">
+      <c r="D57" t="n">
+        <v>24</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>ACLED_all_ZCTA_nb.csv</t>
         </is>
@@ -1242,7 +1415,10 @@
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr">
+      <c r="D58" t="n">
+        <v>12</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousmonth_allZCTA.csv</t>
         </is>
@@ -1256,7 +1432,10 @@
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr">
+      <c r="D59" t="n">
+        <v>22</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousmonth_allZCTA.csv</t>
         </is>
@@ -1270,7 +1449,10 @@
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr">
+      <c r="D60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1284,7 +1466,10 @@
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr">
+      <c r="D61" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1298,7 +1483,10 @@
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr">
+      <c r="D62" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1312,7 +1500,10 @@
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr">
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1326,7 +1517,10 @@
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr">
+      <c r="D64" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1340,7 +1534,10 @@
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr">
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1354,7 +1551,10 @@
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr">
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1368,7 +1568,10 @@
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr">
+      <c r="D67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1382,7 +1585,10 @@
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr">
+      <c r="D68" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1396,7 +1602,10 @@
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr">
+      <c r="D69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1410,7 +1619,10 @@
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr">
+      <c r="D70" t="n">
+        <v>2</v>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1424,7 +1636,10 @@
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr">
+      <c r="D71" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1438,7 +1653,10 @@
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr">
+      <c r="D72" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1452,7 +1670,10 @@
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr">
+      <c r="D73" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1466,7 +1687,10 @@
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr">
+      <c r="D74" t="n">
+        <v>2</v>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1480,7 +1704,10 @@
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr">
+      <c r="D75" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1494,7 +1721,10 @@
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr">
+      <c r="D76" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1508,7 +1738,10 @@
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr">
+      <c r="D77" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1522,7 +1755,10 @@
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr">
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1536,7 +1772,10 @@
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr">
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1550,7 +1789,10 @@
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr">
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
+      <c r="E80" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1564,7 +1806,10 @@
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr">
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1578,7 +1823,10 @@
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr">
+      <c r="D82" t="n">
+        <v>761</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1592,7 +1840,10 @@
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr">
+      <c r="D83" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1606,7 +1857,10 @@
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr">
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1620,7 +1874,10 @@
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr">
+      <c r="D85" t="n">
+        <v>12</v>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1634,7 +1891,10 @@
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr">
+      <c r="D86" t="n">
+        <v>12</v>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1648,7 +1908,10 @@
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr">
+      <c r="D87" t="n">
+        <v>12</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1662,7 +1925,10 @@
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr">
+      <c r="D88" t="n">
+        <v>12</v>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1676,7 +1942,10 @@
       </c>
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr">
+      <c r="D89" t="n">
+        <v>12</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1690,7 +1959,10 @@
       </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr">
+      <c r="D90" t="n">
+        <v>12</v>
+      </c>
+      <c r="E90" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1704,7 +1976,10 @@
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr">
+      <c r="D91" t="n">
+        <v>12</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1718,7 +1993,10 @@
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr">
+      <c r="D92" t="n">
+        <v>12</v>
+      </c>
+      <c r="E92" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1732,7 +2010,10 @@
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr">
+      <c r="D93" t="n">
+        <v>12</v>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1746,7 +2027,10 @@
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr">
+      <c r="D94" t="n">
+        <v>12</v>
+      </c>
+      <c r="E94" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1760,7 +2044,10 @@
       </c>
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr">
+      <c r="D95" t="n">
+        <v>12</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1774,7 +2061,10 @@
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr">
+      <c r="D96" t="n">
+        <v>12</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1788,7 +2078,10 @@
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr">
+      <c r="D97" t="n">
+        <v>12</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1802,7 +2095,10 @@
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr">
+      <c r="D98" t="n">
+        <v>12</v>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1816,7 +2112,10 @@
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr">
+      <c r="D99" t="n">
+        <v>12</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1830,7 +2129,10 @@
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr">
+      <c r="D100" t="n">
+        <v>12</v>
+      </c>
+      <c r="E100" t="inlineStr">
         <is>
           <t>ACLED_Events_21_Clean.csv</t>
         </is>
@@ -1844,7 +2146,10 @@
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr">
+      <c r="D101" t="n">
+        <v>1642</v>
+      </c>
+      <c r="E101" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1858,7 +2163,10 @@
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr">
+      <c r="D102" t="n">
+        <v>1570</v>
+      </c>
+      <c r="E102" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1872,7 +2180,10 @@
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr">
+      <c r="D103" t="n">
+        <v>1833</v>
+      </c>
+      <c r="E103" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1886,7 +2197,10 @@
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr">
+      <c r="D104" t="n">
+        <v>1829</v>
+      </c>
+      <c r="E104" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1900,7 +2214,10 @@
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr">
+      <c r="D105" t="n">
+        <v>3</v>
+      </c>
+      <c r="E105" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1914,7 +2231,10 @@
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr">
+      <c r="D106" t="n">
+        <v>1572</v>
+      </c>
+      <c r="E106" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1928,7 +2248,10 @@
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr">
+      <c r="D107" t="n">
+        <v>418</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1942,7 +2265,10 @@
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr">
+      <c r="D108" t="n">
+        <v>1701</v>
+      </c>
+      <c r="E108" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1956,7 +2282,10 @@
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr">
+      <c r="D109" t="n">
+        <v>1723</v>
+      </c>
+      <c r="E109" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1970,7 +2299,10 @@
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr">
+      <c r="D110" t="n">
+        <v>1759</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1984,7 +2316,10 @@
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr">
+      <c r="D111" t="n">
+        <v>1736</v>
+      </c>
+      <c r="E111" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -1998,7 +2333,10 @@
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr">
+      <c r="D112" t="n">
+        <v>1559</v>
+      </c>
+      <c r="E112" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2012,7 +2350,10 @@
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr">
+      <c r="D113" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E113" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2026,7 +2367,10 @@
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr"/>
-      <c r="D114" t="inlineStr">
+      <c r="D114" t="n">
+        <v>995</v>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2040,7 +2384,10 @@
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr">
+      <c r="D115" t="n">
+        <v>841</v>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2054,7 +2401,10 @@
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr">
+      <c r="D116" t="n">
+        <v>1427</v>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2068,7 +2418,10 @@
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr">
+      <c r="D117" t="n">
+        <v>1285</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2082,7 +2435,10 @@
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr">
+      <c r="D118" t="n">
+        <v>1632</v>
+      </c>
+      <c r="E118" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>

</xml_diff>

<commit_message>
fix codebook column names
</commit_message>
<xml_diff>
--- a/4_Documentation/codebook.xlsx
+++ b/4_Documentation/codebook.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,20 +436,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>var_label</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>var_encoding</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>var_level</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>var_length</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
@@ -463,10 +468,11 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
         <v>761</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -480,10 +486,11 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
         <v>124</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -497,10 +504,11 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -514,10 +522,11 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -531,10 +540,11 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -548,10 +558,11 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -565,10 +576,11 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -582,10 +594,11 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Subevent_22.csv</t>
         </is>
@@ -599,10 +612,11 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="n">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -616,10 +630,11 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
         <v>1798</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -633,10 +648,11 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="n">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
         <v>1798</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -650,10 +666,11 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="n">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -667,10 +684,11 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -684,10 +702,11 @@
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="n">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -701,10 +720,11 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="n">
         <v>1798</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -718,10 +738,11 @@
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="n">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
         <v>1331</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -735,10 +756,11 @@
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="n">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
         <v>1798</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -752,10 +774,11 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="n">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
         <v>1798</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -769,10 +792,11 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="n">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -786,10 +810,11 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="n">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
         <v>1798</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -803,10 +828,11 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="n">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
         <v>1761</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>NeighbouringZCTAs.csv</t>
         </is>
@@ -820,10 +846,11 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="n">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
         <v>12</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -837,10 +864,11 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="n">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
         <v>47</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -854,10 +882,11 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="n">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
         <v>19</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousyear_allZCTA.csv</t>
         </is>
@@ -871,10 +900,11 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="n">
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
         <v>292</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -888,10 +918,11 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="n">
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
         <v>1</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -905,10 +936,11 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -922,10 +954,11 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="n">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
         <v>3</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -939,10 +972,11 @@
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="n">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
         <v>3</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -956,10 +990,11 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="n">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
         <v>6</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -973,10 +1008,11 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="n">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
         <v>7</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -990,10 +1026,11 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="n">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
         <v>327</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1007,10 +1044,11 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="n">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
         <v>5</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1024,10 +1062,11 @@
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="n">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
         <v>4</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1041,10 +1080,11 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="n">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
         <v>11</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1058,10 +1098,11 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="n">
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
         <v>5</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1075,10 +1116,11 @@
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="n">
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
         <v>10</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1092,10 +1134,11 @@
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="n">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
         <v>1</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1109,10 +1152,11 @@
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="n">
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
         <v>1</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1126,10 +1170,11 @@
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="n">
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
         <v>1</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1143,10 +1188,11 @@
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="n">
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
         <v>1</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1160,10 +1206,11 @@
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="n">
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
         <v>1</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1177,10 +1224,11 @@
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="n">
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
         <v>0</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1194,10 +1242,11 @@
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="n">
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
         <v>127</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1211,10 +1260,11 @@
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="n">
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="n">
         <v>125</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1228,10 +1278,11 @@
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="n">
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
         <v>126</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1245,10 +1296,11 @@
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="n">
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
         <v>3</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1262,10 +1314,11 @@
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="n">
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
         <v>304</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1279,10 +1332,11 @@
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" t="n">
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="n">
         <v>15</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1296,10 +1350,11 @@
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
-      <c r="D51" t="n">
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="n">
         <v>761</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1313,10 +1368,11 @@
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
-      <c r="D52" t="n">
-        <v>2</v>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1330,10 +1386,11 @@
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
-      <c r="D53" t="n">
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
         <v>138</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1347,10 +1404,11 @@
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
-      <c r="D54" t="n">
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="n">
         <v>144</v>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1364,10 +1422,11 @@
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="n">
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
         <v>124</v>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>joined_ACLED_ZIP_22_PA.csv</t>
         </is>
@@ -1381,10 +1440,11 @@
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
-      <c r="D56" t="n">
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
         <v>23</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>ACLED_all_ZCTA_nb.csv</t>
         </is>
@@ -1398,10 +1458,11 @@
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
-      <c r="D57" t="n">
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
         <v>24</v>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>ACLED_all_ZCTA_nb.csv</t>
         </is>
@@ -1415,10 +1476,11 @@
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
-      <c r="D58" t="n">
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
         <v>12</v>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousmonth_allZCTA.csv</t>
         </is>
@@ -1432,10 +1494,11 @@
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
-      <c r="D59" t="n">
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="n">
         <v>22</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>ACLED_conflict_previousmonth_allZCTA.csv</t>
         </is>
@@ -1449,10 +1512,11 @@
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
-      <c r="D60" t="n">
-        <v>2</v>
-      </c>
-      <c r="E60" t="inlineStr">
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1466,10 +1530,11 @@
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
-      <c r="D61" t="n">
-        <v>2</v>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1483,10 +1548,11 @@
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
-      <c r="D62" t="n">
-        <v>2</v>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1500,10 +1566,11 @@
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
-      <c r="D63" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1517,10 +1584,11 @@
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
-      <c r="D64" t="n">
-        <v>2</v>
-      </c>
-      <c r="E64" t="inlineStr">
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1534,10 +1602,11 @@
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
-      <c r="D65" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" t="inlineStr">
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1551,10 +1620,11 @@
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
-      <c r="D66" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" t="inlineStr">
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1568,10 +1638,11 @@
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
-      <c r="D67" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" t="inlineStr">
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1585,10 +1656,11 @@
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
-      <c r="D68" t="n">
-        <v>2</v>
-      </c>
-      <c r="E68" t="inlineStr">
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>2</v>
+      </c>
+      <c r="F68" t="inlineStr">
         <is>
           <t>ACLED_ZIP_Actor_22.csv</t>
         </is>
@@ -1602,10 +1674,11 @@
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
-      <c r="D69" t="n">
-        <v>2</v>
-      </c>
-      <c r="E69" t="inlineStr">
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1619,10 +1692,11 @@
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
-      <c r="D70" t="n">
-        <v>2</v>
-      </c>
-      <c r="E70" t="inlineStr">
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1636,10 +1710,11 @@
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
-      <c r="D71" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1653,10 +1728,11 @@
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
-      <c r="D72" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" t="inlineStr">
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1670,10 +1746,11 @@
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
-      <c r="D73" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" t="inlineStr">
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1687,10 +1764,11 @@
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
-      <c r="D74" t="n">
-        <v>2</v>
-      </c>
-      <c r="E74" t="inlineStr">
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1704,10 +1782,11 @@
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
-      <c r="D75" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" t="inlineStr">
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1721,10 +1800,11 @@
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
-      <c r="D76" t="n">
-        <v>2</v>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1738,10 +1818,11 @@
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
-      <c r="D77" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1755,10 +1836,11 @@
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
-      <c r="D78" t="n">
-        <v>2</v>
-      </c>
-      <c r="E78" t="inlineStr">
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1772,10 +1854,11 @@
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
-      <c r="D79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" t="inlineStr">
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1789,10 +1872,11 @@
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
-      <c r="D80" t="n">
-        <v>2</v>
-      </c>
-      <c r="E80" t="inlineStr">
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1806,10 +1890,11 @@
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
-      <c r="D81" t="n">
-        <v>2</v>
-      </c>
-      <c r="E81" t="inlineStr">
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="inlineStr">
         <is>
           <t>ACLED_conflict_all_ZCTA.csv</t>
         </is>
@@ -1823,10 +1908,11 @@
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
-      <c r="D82" t="n">
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="n">
         <v>761</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1840,10 +1926,11 @@
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
-      <c r="D83" t="n">
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="n">
         <v>4</v>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1857,10 +1944,11 @@
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
-      <c r="D84" t="n">
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
         <v>4</v>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>topics.csv</t>
         </is>
@@ -1874,10 +1962,11 @@
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
-      <c r="D85" t="n">
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
         <v>12</v>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1891,10 +1980,11 @@
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr"/>
-      <c r="D86" t="n">
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
         <v>12</v>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1908,10 +1998,11 @@
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr"/>
-      <c r="D87" t="n">
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
         <v>12</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1925,10 +2016,11 @@
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr"/>
-      <c r="D88" t="n">
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="n">
         <v>12</v>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1942,10 +2034,11 @@
       </c>
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr"/>
-      <c r="D89" t="n">
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="n">
         <v>12</v>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1959,10 +2052,11 @@
       </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr"/>
-      <c r="D90" t="n">
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
         <v>12</v>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1976,10 +2070,11 @@
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr"/>
-      <c r="D91" t="n">
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="n">
         <v>12</v>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -1993,10 +2088,11 @@
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr"/>
-      <c r="D92" t="n">
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
         <v>12</v>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2010,10 +2106,11 @@
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr"/>
-      <c r="D93" t="n">
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="n">
         <v>12</v>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2027,10 +2124,11 @@
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr"/>
-      <c r="D94" t="n">
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="n">
         <v>12</v>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2044,10 +2142,11 @@
       </c>
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr"/>
-      <c r="D95" t="n">
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
         <v>12</v>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="F95" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2061,10 +2160,11 @@
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr"/>
-      <c r="D96" t="n">
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
         <v>12</v>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="F96" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2078,10 +2178,11 @@
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr"/>
-      <c r="D97" t="n">
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="n">
         <v>12</v>
       </c>
-      <c r="E97" t="inlineStr">
+      <c r="F97" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2095,10 +2196,11 @@
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr"/>
-      <c r="D98" t="n">
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="n">
         <v>12</v>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="F98" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2112,10 +2214,11 @@
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
-      <c r="D99" t="n">
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="n">
         <v>12</v>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="F99" t="inlineStr">
         <is>
           <t>All_NewsTopic_Features.csv</t>
         </is>
@@ -2129,10 +2232,11 @@
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr"/>
-      <c r="D100" t="n">
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="n">
         <v>12</v>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>ACLED_Events_21_Clean.csv</t>
         </is>
@@ -2146,10 +2250,11 @@
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr"/>
-      <c r="D101" t="n">
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="n">
         <v>1642</v>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="F101" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2163,10 +2268,11 @@
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr"/>
-      <c r="D102" t="n">
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="n">
         <v>1570</v>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2180,10 +2286,11 @@
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr"/>
-      <c r="D103" t="n">
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="n">
         <v>1833</v>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="F103" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2197,10 +2304,11 @@
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr"/>
-      <c r="D104" t="n">
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="n">
         <v>1829</v>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="F104" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2214,10 +2322,11 @@
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
-      <c r="D105" t="n">
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="n">
         <v>3</v>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="F105" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2231,10 +2340,11 @@
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr"/>
-      <c r="D106" t="n">
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="n">
         <v>1572</v>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="F106" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2248,10 +2358,11 @@
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr"/>
-      <c r="D107" t="n">
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="n">
         <v>418</v>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="F107" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2265,10 +2376,11 @@
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr"/>
-      <c r="D108" t="n">
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="n">
         <v>1701</v>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="F108" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2282,10 +2394,11 @@
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr"/>
-      <c r="D109" t="n">
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="n">
         <v>1723</v>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2299,10 +2412,11 @@
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr"/>
-      <c r="D110" t="n">
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="n">
         <v>1759</v>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2316,10 +2430,11 @@
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr"/>
-      <c r="D111" t="n">
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="n">
         <v>1736</v>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="F111" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2333,10 +2448,11 @@
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr"/>
-      <c r="D112" t="n">
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="n">
         <v>1559</v>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="F112" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2350,10 +2466,11 @@
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr"/>
-      <c r="D113" t="n">
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="n">
         <v>1105</v>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="F113" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2367,10 +2484,11 @@
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr"/>
-      <c r="D114" t="n">
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="n">
         <v>995</v>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="F114" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2384,10 +2502,11 @@
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr"/>
-      <c r="D115" t="n">
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="n">
         <v>841</v>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="F115" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2401,10 +2520,11 @@
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr"/>
-      <c r="D116" t="n">
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="n">
         <v>1427</v>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="F116" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2418,10 +2538,11 @@
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr"/>
-      <c r="D117" t="n">
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="n">
         <v>1285</v>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="F117" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>
@@ -2435,10 +2556,11 @@
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr"/>
-      <c r="D118" t="n">
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="n">
         <v>1632</v>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="F118" t="inlineStr">
         <is>
           <t>All_SocDem_Features.csv</t>
         </is>

</xml_diff>